<commit_message>
update the budget_method_templete as per client requirements
</commit_message>
<xml_diff>
--- a/data/Budget_Method_templete.xlsx
+++ b/data/Budget_Method_templete.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tauhid Hasan\Desktop\idalindvall\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC2F51FB-91A2-43A2-BCFA-FF9474680869}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FD46F2-308B-4313-BAFD-E4FC8F39CDBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
     <sheet name="Net Position Snapshot" sheetId="4" r:id="rId4"/>
     <sheet name="Monthly Activation" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -634,7 +634,7 @@
     <numFmt numFmtId="164" formatCode="#,##0&quot; kr&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -652,11 +652,6 @@
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Lato"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
@@ -803,21 +798,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -841,212 +822,218 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="74">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+  <cellXfs count="76">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="1" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1063,10 +1050,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1265,6 +1248,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{65270B96-538E-4F1F-A608-DC67382166DA}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;02faa678-a308-4b4e-bb71-435cb0214da2&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F1000"/>
@@ -1284,24 +1289,24 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="54"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
     </row>
     <row r="4" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1320,14 +1325,14 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
     </row>
     <row r="7" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -1338,14 +1343,14 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="57" t="s">
+      <c r="A8" s="61" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="53"/>
-      <c r="C8" s="53"/>
-      <c r="D8" s="53"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="54"/>
+      <c r="B8" s="56"/>
+      <c r="C8" s="56"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="56"/>
+      <c r="F8" s="56"/>
     </row>
     <row r="9" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
@@ -1356,20 +1361,20 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="54"/>
+      <c r="B10" s="56"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="59" t="s">
+      <c r="A11" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="54"/>
+      <c r="B11" s="56"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -1384,20 +1389,20 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="60" t="s">
+      <c r="A13" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="54"/>
+      <c r="B13" s="56"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="54"/>
+      <c r="B14" s="56"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="3"/>
@@ -1412,20 +1417,20 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="58" t="s">
+      <c r="A16" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="54"/>
+      <c r="B16" s="56"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="59" t="s">
+      <c r="A17" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="54"/>
+      <c r="B17" s="56"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -1440,20 +1445,20 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="60" t="s">
+      <c r="A19" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="54"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="61" t="s">
+      <c r="A20" s="65" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="54"/>
+      <c r="B20" s="56"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
@@ -1476,14 +1481,14 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="57" t="s">
+      <c r="A23" s="61" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="53"/>
-      <c r="C23" s="53"/>
-      <c r="D23" s="53"/>
-      <c r="E23" s="53"/>
-      <c r="F23" s="54"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
     </row>
     <row r="24" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
@@ -1494,20 +1499,20 @@
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="62" t="s">
+      <c r="A25" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="54"/>
+      <c r="B25" s="56"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="61" t="s">
+      <c r="A26" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="54"/>
+      <c r="B26" s="56"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="3"/>
@@ -1522,20 +1527,20 @@
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="65" t="s">
+      <c r="A28" s="66" t="s">
         <v>15</v>
       </c>
-      <c r="B28" s="54"/>
+      <c r="B28" s="56"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="59" t="s">
+      <c r="A29" s="55" t="s">
         <v>16</v>
       </c>
-      <c r="B29" s="54"/>
+      <c r="B29" s="56"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
@@ -1550,20 +1555,20 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="62" t="s">
+      <c r="A31" s="60" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="54"/>
+      <c r="B31" s="56"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
     </row>
     <row r="32" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="61" t="s">
+      <c r="A32" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="B32" s="54"/>
+      <c r="B32" s="56"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
@@ -1578,20 +1583,20 @@
       <c r="F33" s="2"/>
     </row>
     <row r="34" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="65" t="s">
+      <c r="A34" s="66" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="54"/>
+      <c r="B34" s="56"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
     </row>
     <row r="35" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="59" t="s">
+      <c r="A35" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="54"/>
+      <c r="B35" s="56"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -1606,20 +1611,20 @@
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="62" t="s">
+      <c r="A37" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="B37" s="54"/>
+      <c r="B37" s="56"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
     </row>
     <row r="38" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="61" t="s">
+      <c r="A38" s="65" t="s">
         <v>22</v>
       </c>
-      <c r="B38" s="54"/>
+      <c r="B38" s="56"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
@@ -1642,14 +1647,14 @@
       <c r="F40" s="2"/>
     </row>
     <row r="41" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="63" t="s">
+      <c r="A41" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="B41" s="53"/>
-      <c r="C41" s="53"/>
-      <c r="D41" s="53"/>
-      <c r="E41" s="53"/>
-      <c r="F41" s="54"/>
+      <c r="B41" s="56"/>
+      <c r="C41" s="56"/>
+      <c r="D41" s="56"/>
+      <c r="E41" s="56"/>
+      <c r="F41" s="56"/>
     </row>
     <row r="42" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
@@ -1663,11 +1668,11 @@
       <c r="A43" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="B43" s="53"/>
-      <c r="C43" s="53"/>
-      <c r="D43" s="53"/>
-      <c r="E43" s="53"/>
-      <c r="F43" s="54"/>
+      <c r="B43" s="56"/>
+      <c r="C43" s="56"/>
+      <c r="D43" s="56"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="56"/>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="45" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2628,31 +2633,31 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A43:F43"/>
     <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
     <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
     <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A37:B37"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A23:F23"/>
     <mergeCell ref="A8:F8"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A6:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2679,24 +2684,24 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="54"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
     </row>
     <row r="4" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2715,14 +2720,14 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
     </row>
     <row r="7" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -2741,30 +2746,30 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="61" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="53"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="54"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="66" t="s">
+      <c r="A10" s="69" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="54"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
     </row>
     <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="38"/>
+      <c r="B11" s="47"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -2774,7 +2779,7 @@
       <c r="A12" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="39"/>
+      <c r="B12" s="48"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -2784,7 +2789,7 @@
       <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="38"/>
+      <c r="B13" s="47"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
@@ -2794,7 +2799,7 @@
       <c r="A14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="40">
+      <c r="B14" s="6">
         <f>SUM(B11:B13)</f>
         <v>0</v>
       </c>
@@ -2812,24 +2817,24 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="57" t="s">
+      <c r="A16" s="61" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="53"/>
-      <c r="F16" s="54"/>
+      <c r="B16" s="56"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="56"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="66" t="s">
+      <c r="A17" s="69" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="54"/>
+      <c r="B17" s="56"/>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="56"/>
     </row>
     <row r="18" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
@@ -2859,12 +2864,12 @@
       <c r="C19" s="13">
         <v>0.6</v>
       </c>
-      <c r="D19" s="41">
+      <c r="D19" s="38">
         <f>IFERROR(C19*B14,0)</f>
         <v>0</v>
       </c>
       <c r="E19" s="14" t="str">
-        <f t="shared" ref="E19:E22" si="0">IF(C19="","Enter %",IF(C19&gt;0,"Allocated","Not set"))</f>
+        <f>IF(C19="","Enter %",IF(C19&gt;0,"Allocated","Not set"))</f>
         <v>Allocated</v>
       </c>
       <c r="F19" s="3"/>
@@ -2879,12 +2884,12 @@
       <c r="C20" s="17">
         <v>0.1</v>
       </c>
-      <c r="D20" s="44">
+      <c r="D20" s="40">
         <f>IFERROR(C20*B14,0)</f>
         <v>0</v>
       </c>
       <c r="E20" s="18" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C20="","Enter %",IF(C20&gt;0,"Allocated","Not set"))</f>
         <v>Allocated</v>
       </c>
       <c r="F20" s="2"/>
@@ -2899,12 +2904,12 @@
       <c r="C21" s="13">
         <v>0.1</v>
       </c>
-      <c r="D21" s="41">
+      <c r="D21" s="38">
         <f>IFERROR(C21*B14,0)</f>
         <v>0</v>
       </c>
       <c r="E21" s="14" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C21="","Enter %",IF(C21&gt;0,"Allocated","Not set"))</f>
         <v>Allocated</v>
       </c>
       <c r="F21" s="3"/>
@@ -2917,14 +2922,15 @@
         <v>46</v>
       </c>
       <c r="C22" s="17">
-        <v>0.2</v>
-      </c>
-      <c r="D22" s="44">
+        <f>1-C19-C20-C21</f>
+        <v>0.20000000000000004</v>
+      </c>
+      <c r="D22" s="40">
         <f>IFERROR(C22*B14,0)</f>
         <v>0</v>
       </c>
       <c r="E22" s="18" t="str">
-        <f t="shared" si="0"/>
+        <f>IF(C22="","Enter %",IF(C22&gt;0,"Allocated","Not set"))</f>
         <v>Allocated</v>
       </c>
       <c r="F22" s="2"/>
@@ -2962,39 +2968,39 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="53"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="53"/>
-      <c r="F26" s="54"/>
+      <c r="B26" s="56"/>
+      <c r="C26" s="56"/>
+      <c r="D26" s="56"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="56"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="66" t="s">
+      <c r="A27" s="69" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="53"/>
-      <c r="C27" s="53"/>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="54"/>
+      <c r="B27" s="56"/>
+      <c r="C27" s="56"/>
+      <c r="D27" s="56"/>
+      <c r="E27" s="56"/>
+      <c r="F27" s="56"/>
     </row>
     <row r="28" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="41">
+      <c r="B28" s="38">
         <f>'Irregular Expense System'!B45</f>
-        <v>7083.3333333333339</v>
+        <v>0</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28" s="68" t="s">
         <v>51</v>
       </c>
-      <c r="E28" s="53"/>
-      <c r="F28" s="54"/>
+      <c r="E28" s="56"/>
+      <c r="F28" s="56"/>
     </row>
     <row r="29" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
@@ -3005,84 +3011,84 @@
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="57" t="s">
+      <c r="A30" s="61" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
-      <c r="E30" s="53"/>
-      <c r="F30" s="54"/>
+      <c r="B30" s="56"/>
+      <c r="C30" s="56"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="66" t="s">
+      <c r="A31" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="54"/>
+      <c r="B31" s="56"/>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
     </row>
     <row r="32" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="43">
-        <f t="shared" ref="B32:B34" si="1">D20</f>
+      <c r="B32" s="39">
+        <f>D20</f>
         <v>0</v>
       </c>
-      <c r="C32" s="67" t="s">
+      <c r="C32" s="70" t="s">
         <v>55</v>
       </c>
-      <c r="D32" s="53"/>
-      <c r="E32" s="53"/>
-      <c r="F32" s="54"/>
+      <c r="D32" s="56"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="56"/>
     </row>
     <row r="33" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="43">
-        <f t="shared" si="1"/>
+      <c r="B33" s="39">
+        <f>D21</f>
         <v>0</v>
       </c>
       <c r="C33" s="68" t="s">
         <v>55</v>
       </c>
-      <c r="D33" s="53"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="54"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="56"/>
     </row>
     <row r="34" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B34" s="43">
-        <f t="shared" si="1"/>
+      <c r="B34" s="39">
+        <f>D22</f>
         <v>0</v>
       </c>
-      <c r="C34" s="67" t="s">
+      <c r="C34" s="70" t="s">
         <v>58</v>
       </c>
-      <c r="D34" s="53"/>
-      <c r="E34" s="53"/>
-      <c r="F34" s="54"/>
+      <c r="D34" s="56"/>
+      <c r="E34" s="56"/>
+      <c r="F34" s="56"/>
     </row>
     <row r="35" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="43">
+      <c r="B35" s="39">
         <f>B28</f>
-        <v>7083.3333333333339</v>
+        <v>0</v>
       </c>
       <c r="C35" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="D35" s="53"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="54"/>
+      <c r="D35" s="56"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
     </row>
     <row r="36" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
@@ -3096,11 +3102,11 @@
       <c r="A37" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="B37" s="53"/>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="53"/>
-      <c r="F37" s="54"/>
+      <c r="B37" s="56"/>
+      <c r="C37" s="56"/>
+      <c r="D37" s="56"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
     </row>
     <row r="38" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4067,23 +4073,23 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="C35:F35"/>
     <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="A37:F37"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A6:F6"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -4112,24 +4118,24 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="57" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="54"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
     </row>
     <row r="4" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -4148,14 +4154,14 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
     </row>
     <row r="7" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -4192,25 +4198,25 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="57" t="s">
+      <c r="A10" s="61" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="54"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
     </row>
     <row r="11" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B11" s="42">
-        <v>6000</v>
-      </c>
-      <c r="C11" s="41">
-        <f t="shared" ref="C11:C13" si="0">IFERROR(B11/12,0)</f>
-        <v>500</v>
+      <c r="B11" s="49">
+        <v>0</v>
+      </c>
+      <c r="C11" s="38">
+        <f>IFERROR(B11/12,0)</f>
+        <v>0</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="22" t="s">
@@ -4222,9 +4228,11 @@
       <c r="A12" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="44">
-        <f t="shared" si="0"/>
+      <c r="B12" s="50">
+        <v>0</v>
+      </c>
+      <c r="C12" s="40">
+        <f>IFERROR(B12/12,0)</f>
         <v>0</v>
       </c>
       <c r="D12" s="5"/>
@@ -4237,9 +4245,11 @@
       <c r="A13" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="41">
-        <f t="shared" si="0"/>
+      <c r="B13" s="49">
+        <v>0</v>
+      </c>
+      <c r="C13" s="38">
+        <f>IFERROR(B13/12,0)</f>
         <v>0</v>
       </c>
       <c r="D13" s="4"/>
@@ -4250,29 +4260,31 @@
     </row>
     <row r="14" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
+      <c r="B14" s="41"/>
+      <c r="C14" s="41"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="57" t="s">
+      <c r="A15" s="61" t="s">
         <v>73</v>
       </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="54"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
     </row>
     <row r="16" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B16" s="43"/>
-      <c r="C16" s="44">
-        <f t="shared" ref="C16:C19" si="1">IFERROR(B16/12,0)</f>
+      <c r="B16" s="50">
+        <v>0</v>
+      </c>
+      <c r="C16" s="40">
+        <f>IFERROR(B16/12,0)</f>
         <v>0</v>
       </c>
       <c r="D16" s="5"/>
@@ -4285,9 +4297,11 @@
       <c r="A17" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="42"/>
-      <c r="C17" s="41">
-        <f t="shared" si="1"/>
+      <c r="B17" s="49">
+        <v>0</v>
+      </c>
+      <c r="C17" s="38">
+        <f>IFERROR(B17/12,0)</f>
         <v>0</v>
       </c>
       <c r="D17" s="4"/>
@@ -4300,9 +4314,11 @@
       <c r="A18" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B18" s="43"/>
-      <c r="C18" s="44">
-        <f t="shared" si="1"/>
+      <c r="B18" s="50">
+        <v>0</v>
+      </c>
+      <c r="C18" s="40">
+        <f>IFERROR(B18/12,0)</f>
         <v>0</v>
       </c>
       <c r="D18" s="5"/>
@@ -4315,9 +4331,11 @@
       <c r="A19" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="42"/>
-      <c r="C19" s="41">
-        <f t="shared" si="1"/>
+      <c r="B19" s="49">
+        <v>0</v>
+      </c>
+      <c r="C19" s="38">
+        <f>IFERROR(B19/12,0)</f>
         <v>0</v>
       </c>
       <c r="D19" s="4"/>
@@ -4328,32 +4346,32 @@
     </row>
     <row r="20" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="45"/>
-      <c r="C20" s="45"/>
+      <c r="B20" s="41"/>
+      <c r="C20" s="41"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
     <row r="21" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="57" t="s">
+      <c r="A21" s="61" t="s">
         <v>79</v>
       </c>
-      <c r="B21" s="53"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="53"/>
-      <c r="F21" s="54"/>
+      <c r="B21" s="56"/>
+      <c r="C21" s="56"/>
+      <c r="D21" s="56"/>
+      <c r="E21" s="56"/>
+      <c r="F21" s="56"/>
     </row>
     <row r="22" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B22" s="43">
-        <v>3000</v>
-      </c>
-      <c r="C22" s="44">
-        <f t="shared" ref="C22:C24" si="2">IFERROR(B22/12,0)</f>
-        <v>250</v>
+      <c r="B22" s="50">
+        <v>0</v>
+      </c>
+      <c r="C22" s="40">
+        <f>IFERROR(B22/12,0)</f>
+        <v>0</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="23" t="s">
@@ -4365,12 +4383,12 @@
       <c r="A23" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="42">
-        <v>6000</v>
-      </c>
-      <c r="C23" s="41">
-        <f t="shared" si="2"/>
-        <v>500</v>
+      <c r="B23" s="49">
+        <v>0</v>
+      </c>
+      <c r="C23" s="38">
+        <f>IFERROR(B23/12,0)</f>
+        <v>0</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="22" t="s">
@@ -4382,12 +4400,10 @@
       <c r="A24" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B24" s="43">
-        <v>10000</v>
-      </c>
-      <c r="C24" s="44">
-        <f t="shared" si="2"/>
-        <v>833.33333333333337</v>
+      <c r="B24" s="50"/>
+      <c r="C24" s="40">
+        <f>IFERROR(B24/12,0)</f>
+        <v>0</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="23" t="s">
@@ -4397,32 +4413,32 @@
     </row>
     <row r="25" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="45"/>
-      <c r="C25" s="45"/>
+      <c r="B25" s="41"/>
+      <c r="C25" s="41"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="57" t="s">
+      <c r="A26" s="61" t="s">
         <v>84</v>
       </c>
-      <c r="B26" s="53"/>
-      <c r="C26" s="53"/>
-      <c r="D26" s="53"/>
-      <c r="E26" s="53"/>
-      <c r="F26" s="54"/>
+      <c r="B26" s="56"/>
+      <c r="C26" s="56"/>
+      <c r="D26" s="56"/>
+      <c r="E26" s="56"/>
+      <c r="F26" s="56"/>
     </row>
     <row r="27" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B27" s="42">
-        <v>40000</v>
-      </c>
-      <c r="C27" s="41">
-        <f t="shared" ref="C27:C29" si="3">IFERROR(B27/12,0)</f>
-        <v>3333.3333333333335</v>
+      <c r="B27" s="49">
+        <v>0</v>
+      </c>
+      <c r="C27" s="38">
+        <f>IFERROR(B27/12,0)</f>
+        <v>0</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="22" t="s">
@@ -4434,12 +4450,12 @@
       <c r="A28" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B28" s="43">
-        <v>20000</v>
-      </c>
-      <c r="C28" s="44">
-        <f t="shared" si="3"/>
-        <v>1666.6666666666667</v>
+      <c r="B28" s="50">
+        <v>0</v>
+      </c>
+      <c r="C28" s="40">
+        <f>IFERROR(B28/12,0)</f>
+        <v>0</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="23" t="s">
@@ -4451,9 +4467,11 @@
       <c r="A29" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B29" s="42"/>
-      <c r="C29" s="41">
-        <f t="shared" si="3"/>
+      <c r="B29" s="49">
+        <v>0</v>
+      </c>
+      <c r="C29" s="38">
+        <f>IFERROR(B29/12,0)</f>
         <v>0</v>
       </c>
       <c r="D29" s="4"/>
@@ -4471,22 +4489,24 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="57" t="s">
+      <c r="A31" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="54"/>
+      <c r="B31" s="56"/>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
     </row>
     <row r="32" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B32" s="43"/>
-      <c r="C32" s="44">
-        <f t="shared" ref="C32:C34" si="4">IFERROR(B32/12,0)</f>
+      <c r="B32" s="50">
+        <v>0</v>
+      </c>
+      <c r="C32" s="40">
+        <f>IFERROR(B32/12,0)</f>
         <v>0</v>
       </c>
       <c r="D32" s="5"/>
@@ -4499,9 +4519,11 @@
       <c r="A33" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B33" s="42"/>
-      <c r="C33" s="41">
-        <f t="shared" si="4"/>
+      <c r="B33" s="49">
+        <v>0</v>
+      </c>
+      <c r="C33" s="38">
+        <f>IFERROR(B33/12,0)</f>
         <v>0</v>
       </c>
       <c r="D33" s="4"/>
@@ -4514,9 +4536,11 @@
       <c r="A34" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B34" s="43"/>
-      <c r="C34" s="44">
-        <f t="shared" si="4"/>
+      <c r="B34" s="50">
+        <v>0</v>
+      </c>
+      <c r="C34" s="40">
+        <f>IFERROR(B34/12,0)</f>
         <v>0</v>
       </c>
       <c r="D34" s="5"/>
@@ -4534,22 +4558,24 @@
       <c r="F35" s="2"/>
     </row>
     <row r="36" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="57" t="s">
+      <c r="A36" s="61" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="53"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="53"/>
-      <c r="E36" s="53"/>
-      <c r="F36" s="54"/>
+      <c r="B36" s="56"/>
+      <c r="C36" s="56"/>
+      <c r="D36" s="56"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="56"/>
     </row>
     <row r="37" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B37" s="42"/>
-      <c r="C37" s="41">
-        <f t="shared" ref="C37:C39" si="5">IFERROR(B37/12,0)</f>
+      <c r="B37" s="49">
+        <v>0</v>
+      </c>
+      <c r="C37" s="38">
+        <f>IFERROR(B37/12,0)</f>
         <v>0</v>
       </c>
       <c r="D37" s="4"/>
@@ -4562,9 +4588,11 @@
       <c r="A38" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B38" s="43"/>
-      <c r="C38" s="44">
-        <f t="shared" si="5"/>
+      <c r="B38" s="50">
+        <v>0</v>
+      </c>
+      <c r="C38" s="40">
+        <f>IFERROR(B38/12,0)</f>
         <v>0</v>
       </c>
       <c r="D38" s="5"/>
@@ -4577,9 +4605,11 @@
       <c r="A39" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="B39" s="42"/>
-      <c r="C39" s="41">
-        <f t="shared" si="5"/>
+      <c r="B39" s="49">
+        <v>0</v>
+      </c>
+      <c r="C39" s="38">
+        <f>IFERROR(B39/12,0)</f>
         <v>0</v>
       </c>
       <c r="D39" s="4"/>
@@ -4590,8 +4620,8 @@
     </row>
     <row r="40" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2"/>
-      <c r="B40" s="45"/>
-      <c r="C40" s="45"/>
+      <c r="B40" s="41"/>
+      <c r="C40" s="41"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
@@ -4601,14 +4631,14 @@
         <v>97</v>
       </c>
       <c r="B41" s="7"/>
-      <c r="C41" s="46">
-        <f t="shared" ref="C41" si="6">SUM(C11:C39)</f>
-        <v>7083.3333333333339</v>
-      </c>
-      <c r="D41" s="69" t="s">
+      <c r="C41" s="42">
+        <f>SUM(C11:C39)</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="71" t="s">
         <v>98</v>
       </c>
-      <c r="E41" s="54"/>
+      <c r="E41" s="56"/>
       <c r="F41" s="8"/>
     </row>
     <row r="42" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4620,39 +4650,39 @@
       <c r="F42" s="2"/>
     </row>
     <row r="43" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="57" t="s">
+      <c r="A43" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="B43" s="53"/>
-      <c r="C43" s="53"/>
-      <c r="D43" s="53"/>
-      <c r="E43" s="53"/>
-      <c r="F43" s="54"/>
+      <c r="B43" s="56"/>
+      <c r="C43" s="56"/>
+      <c r="D43" s="56"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="56"/>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="66" t="s">
+      <c r="A44" s="69" t="s">
         <v>100</v>
       </c>
-      <c r="B44" s="53"/>
-      <c r="C44" s="53"/>
-      <c r="D44" s="53"/>
-      <c r="E44" s="53"/>
-      <c r="F44" s="54"/>
+      <c r="B44" s="56"/>
+      <c r="C44" s="56"/>
+      <c r="D44" s="56"/>
+      <c r="E44" s="56"/>
+      <c r="F44" s="56"/>
     </row>
     <row r="45" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="B45" s="41">
+      <c r="B45" s="38">
         <f>C41</f>
-        <v>7083.3333333333339</v>
+        <v>0</v>
       </c>
       <c r="C45" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="D45" s="53"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="54"/>
+      <c r="D45" s="56"/>
+      <c r="E45" s="56"/>
+      <c r="F45" s="56"/>
     </row>
     <row r="46" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
@@ -4660,27 +4690,27 @@
       </c>
       <c r="B46" s="24" t="str">
         <f>IF(C41&gt;0,"YES — SURPRISES ENGINEERED OUT","Add your irregular expenses above")</f>
-        <v>YES — SURPRISES ENGINEERED OUT</v>
-      </c>
-      <c r="C46" s="67"/>
-      <c r="D46" s="53"/>
-      <c r="E46" s="53"/>
-      <c r="F46" s="54"/>
+        <v>Add your irregular expenses above</v>
+      </c>
+      <c r="C46" s="70"/>
+      <c r="D46" s="56"/>
+      <c r="E46" s="56"/>
+      <c r="F46" s="56"/>
     </row>
     <row r="47" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B47" s="41">
-        <f>IF(B41&gt;0,12,0)</f>
+      <c r="B47" s="38">
+        <f>IFERROR('Net Position Snapshot'!B12/C41,0)</f>
         <v>0</v>
       </c>
       <c r="C47" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="D47" s="53"/>
-      <c r="E47" s="53"/>
-      <c r="F47" s="54"/>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
     </row>
     <row r="48" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
@@ -4694,11 +4724,11 @@
       <c r="A49" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="B49" s="53"/>
-      <c r="C49" s="53"/>
-      <c r="D49" s="53"/>
-      <c r="E49" s="53"/>
-      <c r="F49" s="54"/>
+      <c r="B49" s="56"/>
+      <c r="C49" s="56"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
     </row>
     <row r="50" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="51" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5653,22 +5683,22 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="C47:F47"/>
     <mergeCell ref="A21:F21"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="C47:F47"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="A15:F15"/>
     <mergeCell ref="A43:F43"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="C46:F46"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -5695,24 +5725,24 @@
       <c r="F1" s="25"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="57" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="54"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
     </row>
     <row r="4" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="25"/>
@@ -5731,14 +5761,14 @@
       <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="63" t="s">
         <v>107</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
     </row>
     <row r="7" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
@@ -5773,33 +5803,35 @@
       <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="57" t="s">
+      <c r="A10" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="54"/>
+      <c r="B10" s="56"/>
+      <c r="C10" s="56"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="66" t="s">
+      <c r="A11" s="69" t="s">
         <v>113</v>
       </c>
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="53"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="54"/>
+      <c r="B11" s="56"/>
+      <c r="C11" s="56"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="56"/>
     </row>
     <row r="12" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B12" s="47"/>
+      <c r="B12" s="51">
+        <v>0</v>
+      </c>
       <c r="C12" s="26" t="str">
         <f>IF(B12="","Enter value",IF(B12&lt;1000,"[ STATUS: CRITICAL ]",IF(B12&lt;5000,"[ STATUS: THIN ]","[ STATUS: ADEQUATE ]")))</f>
-        <v>Enter value</v>
+        <v>[ STATUS: CRITICAL ]</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>115</v>
@@ -5816,30 +5848,32 @@
       <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="57" t="s">
+      <c r="A14" s="61" t="s">
         <v>116</v>
       </c>
-      <c r="B14" s="53"/>
-      <c r="C14" s="53"/>
-      <c r="D14" s="53"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="54"/>
+      <c r="B14" s="56"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="66" t="s">
+      <c r="A15" s="69" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="54"/>
+      <c r="B15" s="56"/>
+      <c r="C15" s="56"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
     </row>
     <row r="16" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B16" s="48"/>
+      <c r="B16" s="52">
+        <v>0</v>
+      </c>
       <c r="C16" s="5"/>
       <c r="D16" s="23"/>
       <c r="E16" s="5"/>
@@ -5849,7 +5883,9 @@
       <c r="A17" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B17" s="47"/>
+      <c r="B17" s="51">
+        <v>0</v>
+      </c>
       <c r="C17" s="4"/>
       <c r="D17" s="22"/>
       <c r="E17" s="4"/>
@@ -5859,7 +5895,9 @@
       <c r="A18" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="48"/>
+      <c r="B18" s="52">
+        <v>0</v>
+      </c>
       <c r="C18" s="5"/>
       <c r="D18" s="23" t="s">
         <v>121</v>
@@ -5871,7 +5909,9 @@
       <c r="A19" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B19" s="47"/>
+      <c r="B19" s="51">
+        <v>0</v>
+      </c>
       <c r="C19" s="4"/>
       <c r="D19" s="22"/>
       <c r="E19" s="4"/>
@@ -5881,7 +5921,7 @@
       <c r="A20" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B20" s="49">
+      <c r="B20" s="45">
         <f>SUM(B16:B19)</f>
         <v>0</v>
       </c>
@@ -5902,30 +5942,32 @@
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="57" t="s">
+      <c r="A22" s="61" t="s">
         <v>124</v>
       </c>
-      <c r="B22" s="53"/>
-      <c r="C22" s="53"/>
-      <c r="D22" s="53"/>
-      <c r="E22" s="53"/>
-      <c r="F22" s="54"/>
+      <c r="B22" s="56"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="56"/>
+      <c r="F22" s="56"/>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="66" t="s">
+      <c r="A23" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="B23" s="53"/>
-      <c r="C23" s="53"/>
-      <c r="D23" s="53"/>
-      <c r="E23" s="53"/>
-      <c r="F23" s="54"/>
+      <c r="B23" s="56"/>
+      <c r="C23" s="56"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
+      <c r="F23" s="56"/>
     </row>
     <row r="24" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B24" s="48"/>
+      <c r="B24" s="52">
+        <v>0</v>
+      </c>
       <c r="C24" s="5"/>
       <c r="D24" s="23" t="s">
         <v>127</v>
@@ -5937,7 +5979,9 @@
       <c r="A25" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="B25" s="47"/>
+      <c r="B25" s="51">
+        <v>0</v>
+      </c>
       <c r="C25" s="4"/>
       <c r="D25" s="22"/>
       <c r="E25" s="4"/>
@@ -5947,7 +5991,9 @@
       <c r="A26" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B26" s="48"/>
+      <c r="B26" s="52">
+        <v>0</v>
+      </c>
       <c r="C26" s="5"/>
       <c r="D26" s="23"/>
       <c r="E26" s="5"/>
@@ -5957,7 +6003,9 @@
       <c r="A27" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="B27" s="47"/>
+      <c r="B27" s="51">
+        <v>0</v>
+      </c>
       <c r="C27" s="4"/>
       <c r="D27" s="22"/>
       <c r="E27" s="4"/>
@@ -5967,7 +6015,9 @@
       <c r="A28" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="B28" s="48"/>
+      <c r="B28" s="52">
+        <v>0</v>
+      </c>
       <c r="C28" s="5"/>
       <c r="D28" s="23"/>
       <c r="E28" s="5"/>
@@ -5977,7 +6027,7 @@
       <c r="A29" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="49">
+      <c r="B29" s="45">
         <f>SUM(B24:B28)</f>
         <v>0</v>
       </c>
@@ -5998,30 +6048,30 @@
       <c r="F30" s="5"/>
     </row>
     <row r="31" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="57" t="s">
+      <c r="A31" s="61" t="s">
         <v>133</v>
       </c>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="54"/>
+      <c r="B31" s="56"/>
+      <c r="C31" s="56"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
     </row>
     <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="66" t="s">
+      <c r="A32" s="69" t="s">
         <v>134</v>
       </c>
-      <c r="B32" s="53"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
-      <c r="E32" s="53"/>
-      <c r="F32" s="54"/>
+      <c r="B32" s="56"/>
+      <c r="C32" s="56"/>
+      <c r="D32" s="56"/>
+      <c r="E32" s="56"/>
+      <c r="F32" s="56"/>
     </row>
     <row r="33" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B33" s="47">
+      <c r="B33" s="43">
         <f>B18</f>
         <v>0</v>
       </c>
@@ -6036,7 +6086,7 @@
       <c r="A34" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B34" s="48">
+      <c r="B34" s="44">
         <f>B24</f>
         <v>0</v>
       </c>
@@ -6051,7 +6101,7 @@
       <c r="A35" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B35" s="50">
+      <c r="B35" s="46">
         <f>B18-B24</f>
         <v>0</v>
       </c>
@@ -6082,11 +6132,11 @@
         <f>IF(OR(B12=0,B20=0),"Enter values above",IF(B12+B20-B29&gt;0,"[ SYSTEM STABLE ]","[ ACTION REQUIRED ]"))</f>
         <v>Enter values above</v>
       </c>
-      <c r="D37" s="70" t="s">
+      <c r="D37" s="72" t="s">
         <v>142</v>
       </c>
-      <c r="E37" s="53"/>
-      <c r="F37" s="54"/>
+      <c r="E37" s="56"/>
+      <c r="F37" s="56"/>
     </row>
     <row r="38" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
@@ -6097,31 +6147,31 @@
       <c r="F38" s="5"/>
     </row>
     <row r="39" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="57" t="s">
+      <c r="A39" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="B39" s="53"/>
-      <c r="C39" s="53"/>
-      <c r="D39" s="53"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="54"/>
+      <c r="B39" s="56"/>
+      <c r="C39" s="56"/>
+      <c r="D39" s="56"/>
+      <c r="E39" s="56"/>
+      <c r="F39" s="56"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="66" t="s">
+      <c r="A40" s="69" t="s">
         <v>144</v>
       </c>
-      <c r="B40" s="53"/>
-      <c r="C40" s="53"/>
-      <c r="D40" s="53"/>
-      <c r="E40" s="53"/>
-      <c r="F40" s="54"/>
+      <c r="B40" s="56"/>
+      <c r="C40" s="56"/>
+      <c r="D40" s="56"/>
+      <c r="E40" s="56"/>
+      <c r="F40" s="56"/>
     </row>
     <row r="41" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>145</v>
       </c>
       <c r="B41" s="33">
-        <f>IFERROR(B12/(B12+(B20-B18)+(B18-B24)),0)</f>
+        <f>IFERROR(B12/(B12+B20),0)</f>
         <v>0</v>
       </c>
       <c r="C41" s="22" t="s">
@@ -6136,7 +6186,7 @@
         <v>146</v>
       </c>
       <c r="B42" s="34">
-        <f>IFERROR((B20-B18)/(B12+(B20-B18)+(B18-B24)),0)</f>
+        <f>IFERROR((B16+B17)/(B12+B20),0)</f>
         <v>0</v>
       </c>
       <c r="C42" s="23" t="s">
@@ -6151,7 +6201,7 @@
         <v>148</v>
       </c>
       <c r="B43" s="33">
-        <f>IFERROR((B18-B24)/(B12+(B20-B18)+(B18-B24)),0)</f>
+        <f>IFERROR((B18-B24)/(B12+B20),0)</f>
         <v>0</v>
       </c>
       <c r="C43" s="22" t="s">
@@ -6181,7 +6231,7 @@
         <v>152</v>
       </c>
       <c r="B45" s="33">
-        <f>IFERROR((B29-B24)/(B12+(B20-B18)+(B18-B24)),0)</f>
+        <f>IFERROR((B25+B26+B27+B28)/(B12+B20),0)</f>
         <v>0</v>
       </c>
       <c r="C45" s="22" t="s">
@@ -6203,11 +6253,11 @@
       <c r="A47" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="B47" s="53"/>
-      <c r="C47" s="53"/>
-      <c r="D47" s="53"/>
-      <c r="E47" s="53"/>
-      <c r="F47" s="54"/>
+      <c r="B47" s="56"/>
+      <c r="C47" s="56"/>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
     </row>
     <row r="48" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -7164,21 +7214,21 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A47:F47"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="D37:F37"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="D37:F37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -7205,24 +7255,24 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52" t="s">
+      <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="55" t="s">
+      <c r="A3" s="57" t="s">
         <v>154</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="53"/>
-      <c r="F3" s="54"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="56"/>
+      <c r="E3" s="56"/>
+      <c r="F3" s="56"/>
     </row>
     <row r="4" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -7241,14 +7291,14 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="63" t="s">
         <v>155</v>
       </c>
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="53"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="56"/>
+      <c r="C6" s="56"/>
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
     </row>
     <row r="7" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -7267,50 +7317,52 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="61" t="s">
         <v>156</v>
       </c>
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
-      <c r="D9" s="53"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="54"/>
+      <c r="B9" s="56"/>
+      <c r="C9" s="56"/>
+      <c r="D9" s="56"/>
+      <c r="E9" s="56"/>
+      <c r="F9" s="56"/>
     </row>
     <row r="10" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="67" t="s">
+      <c r="B10" s="53"/>
+      <c r="C10" s="70" t="s">
         <v>158</v>
       </c>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="54"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
     </row>
     <row r="11" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="B11" s="51"/>
+      <c r="B11" s="54">
+        <v>0</v>
+      </c>
       <c r="C11" s="68" t="s">
         <v>160</v>
       </c>
-      <c r="D11" s="53"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="54"/>
+      <c r="D11" s="56"/>
+      <c r="E11" s="56"/>
+      <c r="F11" s="56"/>
     </row>
     <row r="12" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>161</v>
       </c>
       <c r="B12" s="2"/>
-      <c r="C12" s="67" t="s">
+      <c r="C12" s="70" t="s">
         <v>162</v>
       </c>
-      <c r="D12" s="53"/>
-      <c r="E12" s="53"/>
-      <c r="F12" s="54"/>
+      <c r="D12" s="56"/>
+      <c r="E12" s="56"/>
+      <c r="F12" s="56"/>
     </row>
     <row r="13" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
@@ -7321,14 +7373,14 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="57" t="s">
+      <c r="A14" s="61" t="s">
         <v>163</v>
       </c>
-      <c r="B14" s="53"/>
-      <c r="C14" s="53"/>
-      <c r="D14" s="53"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="54"/>
+      <c r="B14" s="56"/>
+      <c r="C14" s="56"/>
+      <c r="D14" s="56"/>
+      <c r="E14" s="56"/>
+      <c r="F14" s="56"/>
     </row>
     <row r="15" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="30" t="s">
@@ -7338,12 +7390,12 @@
         <f>'Net Position Snapshot'!C37</f>
         <v>Enter values above</v>
       </c>
-      <c r="C15" s="70" t="s">
+      <c r="C15" s="72" t="s">
         <v>165</v>
       </c>
-      <c r="D15" s="53"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="54"/>
+      <c r="D15" s="56"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="56"/>
     </row>
     <row r="16" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
@@ -7354,133 +7406,133 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="57" t="s">
+      <c r="A17" s="61" t="s">
         <v>166</v>
       </c>
-      <c r="B17" s="53"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="53"/>
-      <c r="F17" s="54"/>
+      <c r="B17" s="56"/>
+      <c r="C17" s="56"/>
+      <c r="D17" s="56"/>
+      <c r="E17" s="56"/>
+      <c r="F17" s="56"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="66" t="s">
+      <c r="A18" s="69" t="s">
         <v>167</v>
       </c>
-      <c r="B18" s="53"/>
-      <c r="C18" s="53"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="54"/>
+      <c r="B18" s="56"/>
+      <c r="C18" s="56"/>
+      <c r="D18" s="56"/>
+      <c r="E18" s="56"/>
+      <c r="F18" s="56"/>
     </row>
     <row r="19" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="72" t="s">
+      <c r="A19" s="74" t="s">
         <v>168</v>
       </c>
-      <c r="B19" s="54"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="68" t="s">
         <v>169</v>
       </c>
-      <c r="D19" s="53"/>
-      <c r="E19" s="54"/>
+      <c r="D19" s="56"/>
+      <c r="E19" s="56"/>
       <c r="F19" s="36" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="71" t="s">
+      <c r="A20" s="75" t="s">
         <v>171</v>
       </c>
-      <c r="B20" s="54"/>
-      <c r="C20" s="67" t="s">
+      <c r="B20" s="56"/>
+      <c r="C20" s="70" t="s">
         <v>172</v>
       </c>
-      <c r="D20" s="53"/>
-      <c r="E20" s="54"/>
+      <c r="D20" s="56"/>
+      <c r="E20" s="56"/>
       <c r="F20" s="37" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="72" t="s">
+      <c r="A21" s="74" t="s">
         <v>173</v>
       </c>
-      <c r="B21" s="54"/>
+      <c r="B21" s="56"/>
       <c r="C21" s="68" t="s">
         <v>174</v>
       </c>
-      <c r="D21" s="53"/>
-      <c r="E21" s="54"/>
+      <c r="D21" s="56"/>
+      <c r="E21" s="56"/>
       <c r="F21" s="36" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="71" t="s">
+      <c r="A22" s="75" t="s">
         <v>175</v>
       </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="67" t="s">
+      <c r="B22" s="56"/>
+      <c r="C22" s="70" t="s">
         <v>176</v>
       </c>
-      <c r="D22" s="53"/>
-      <c r="E22" s="54"/>
+      <c r="D22" s="56"/>
+      <c r="E22" s="56"/>
       <c r="F22" s="37" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="72" t="s">
+      <c r="A23" s="74" t="s">
         <v>178</v>
       </c>
-      <c r="B23" s="54"/>
+      <c r="B23" s="56"/>
       <c r="C23" s="68" t="s">
         <v>179</v>
       </c>
-      <c r="D23" s="53"/>
-      <c r="E23" s="54"/>
+      <c r="D23" s="56"/>
+      <c r="E23" s="56"/>
       <c r="F23" s="36" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="71" t="s">
+      <c r="A24" s="75" t="s">
         <v>181</v>
       </c>
-      <c r="B24" s="54"/>
-      <c r="C24" s="67" t="s">
+      <c r="B24" s="56"/>
+      <c r="C24" s="70" t="s">
         <v>182</v>
       </c>
-      <c r="D24" s="53"/>
-      <c r="E24" s="54"/>
+      <c r="D24" s="56"/>
+      <c r="E24" s="56"/>
       <c r="F24" s="37" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="72" t="s">
+      <c r="A25" s="74" t="s">
         <v>184</v>
       </c>
-      <c r="B25" s="54"/>
+      <c r="B25" s="56"/>
       <c r="C25" s="68" t="s">
         <v>185</v>
       </c>
-      <c r="D25" s="53"/>
-      <c r="E25" s="54"/>
+      <c r="D25" s="56"/>
+      <c r="E25" s="56"/>
       <c r="F25" s="36" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="71" t="s">
+      <c r="A26" s="75" t="s">
         <v>187</v>
       </c>
-      <c r="B26" s="54"/>
-      <c r="C26" s="67" t="s">
+      <c r="B26" s="56"/>
+      <c r="C26" s="70" t="s">
         <v>188</v>
       </c>
-      <c r="D26" s="53"/>
-      <c r="E26" s="54"/>
+      <c r="D26" s="56"/>
+      <c r="E26" s="56"/>
       <c r="F26" s="37" t="s">
         <v>189</v>
       </c>
@@ -7494,14 +7546,14 @@
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="57" t="s">
+      <c r="A28" s="61" t="s">
         <v>190</v>
       </c>
-      <c r="B28" s="53"/>
-      <c r="C28" s="53"/>
-      <c r="D28" s="53"/>
-      <c r="E28" s="53"/>
-      <c r="F28" s="54"/>
+      <c r="B28" s="56"/>
+      <c r="C28" s="56"/>
+      <c r="D28" s="56"/>
+      <c r="E28" s="56"/>
+      <c r="F28" s="56"/>
     </row>
     <row r="29" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
@@ -7511,21 +7563,21 @@
       <c r="C29" s="68" t="s">
         <v>192</v>
       </c>
-      <c r="D29" s="53"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="54"/>
+      <c r="D29" s="56"/>
+      <c r="E29" s="56"/>
+      <c r="F29" s="56"/>
     </row>
     <row r="30" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B30" s="2"/>
-      <c r="C30" s="67" t="s">
+      <c r="C30" s="70" t="s">
         <v>194</v>
       </c>
-      <c r="D30" s="53"/>
-      <c r="E30" s="53"/>
-      <c r="F30" s="54"/>
+      <c r="D30" s="56"/>
+      <c r="E30" s="56"/>
+      <c r="F30" s="56"/>
     </row>
     <row r="31" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
@@ -7533,9 +7585,9 @@
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="68"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="54"/>
+      <c r="D31" s="56"/>
+      <c r="E31" s="56"/>
+      <c r="F31" s="56"/>
     </row>
     <row r="32" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
@@ -7549,11 +7601,11 @@
       <c r="A33" s="73" t="s">
         <v>195</v>
       </c>
-      <c r="B33" s="53"/>
-      <c r="C33" s="53"/>
-      <c r="D33" s="53"/>
-      <c r="E33" s="53"/>
-      <c r="F33" s="54"/>
+      <c r="B33" s="56"/>
+      <c r="C33" s="56"/>
+      <c r="D33" s="56"/>
+      <c r="E33" s="56"/>
+      <c r="F33" s="56"/>
     </row>
     <row r="34" spans="1:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
@@ -7567,11 +7619,11 @@
       <c r="A35" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="B35" s="53"/>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="53"/>
-      <c r="F35" s="54"/>
+      <c r="B35" s="56"/>
+      <c r="C35" s="56"/>
+      <c r="D35" s="56"/>
+      <c r="E35" s="56"/>
+      <c r="F35" s="56"/>
     </row>
     <row r="36" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="37" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -8540,39 +8592,39 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C29:F29"/>
     <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="A19:B19"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A14:F14"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C30:F30"/>
     <mergeCell ref="C15:F15"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A6:F6"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="A18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
update excle file, comment unnecessary print and income data
</commit_message>
<xml_diff>
--- a/data/Budget_Method_templete.xlsx
+++ b/data/Budget_Method_templete.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tauhid Hasan\Desktop\idalindvall\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\idalindvall\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FD46F2-308B-4313-BAFD-E4FC8F39CDBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE092FA-4C19-4B6F-B308-9D89663E93F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -974,10 +974,28 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -987,35 +1005,17 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1026,14 +1026,14 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1289,7 +1289,7 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="64" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
@@ -1299,7 +1299,7 @@
       <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="63" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="56"/>
@@ -1325,7 +1325,7 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="67" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="56"/>
@@ -1343,7 +1343,7 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="61" t="s">
+      <c r="A8" s="66" t="s">
         <v>3</v>
       </c>
       <c r="B8" s="56"/>
@@ -1361,7 +1361,7 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="65" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="56"/>
@@ -1371,7 +1371,7 @@
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="55" t="s">
+      <c r="A11" s="58" t="s">
         <v>5</v>
       </c>
       <c r="B11" s="56"/>
@@ -1389,7 +1389,7 @@
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="62" t="s">
+      <c r="A13" s="59" t="s">
         <v>6</v>
       </c>
       <c r="B13" s="56"/>
@@ -1399,7 +1399,7 @@
       <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="65" t="s">
+      <c r="A14" s="57" t="s">
         <v>7</v>
       </c>
       <c r="B14" s="56"/>
@@ -1417,7 +1417,7 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="59" t="s">
+      <c r="A16" s="65" t="s">
         <v>8</v>
       </c>
       <c r="B16" s="56"/>
@@ -1427,7 +1427,7 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="55" t="s">
+      <c r="A17" s="58" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="56"/>
@@ -1445,7 +1445,7 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="62" t="s">
+      <c r="A19" s="59" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="56"/>
@@ -1455,7 +1455,7 @@
       <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="65" t="s">
+      <c r="A20" s="57" t="s">
         <v>11</v>
       </c>
       <c r="B20" s="56"/>
@@ -1481,7 +1481,7 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="61" t="s">
+      <c r="A23" s="66" t="s">
         <v>12</v>
       </c>
       <c r="B23" s="56"/>
@@ -1499,7 +1499,7 @@
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="60" t="s">
+      <c r="A25" s="61" t="s">
         <v>13</v>
       </c>
       <c r="B25" s="56"/>
@@ -1509,7 +1509,7 @@
       <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="65" t="s">
+      <c r="A26" s="57" t="s">
         <v>14</v>
       </c>
       <c r="B26" s="56"/>
@@ -1527,7 +1527,7 @@
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="66" t="s">
+      <c r="A28" s="60" t="s">
         <v>15</v>
       </c>
       <c r="B28" s="56"/>
@@ -1537,7 +1537,7 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="55" t="s">
+      <c r="A29" s="58" t="s">
         <v>16</v>
       </c>
       <c r="B29" s="56"/>
@@ -1555,7 +1555,7 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="60" t="s">
+      <c r="A31" s="61" t="s">
         <v>17</v>
       </c>
       <c r="B31" s="56"/>
@@ -1565,7 +1565,7 @@
       <c r="F31" s="3"/>
     </row>
     <row r="32" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="65" t="s">
+      <c r="A32" s="57" t="s">
         <v>18</v>
       </c>
       <c r="B32" s="56"/>
@@ -1583,7 +1583,7 @@
       <c r="F33" s="2"/>
     </row>
     <row r="34" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="66" t="s">
+      <c r="A34" s="60" t="s">
         <v>19</v>
       </c>
       <c r="B34" s="56"/>
@@ -1593,7 +1593,7 @@
       <c r="F34" s="2"/>
     </row>
     <row r="35" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="55" t="s">
+      <c r="A35" s="58" t="s">
         <v>20</v>
       </c>
       <c r="B35" s="56"/>
@@ -1611,7 +1611,7 @@
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="60" t="s">
+      <c r="A37" s="61" t="s">
         <v>21</v>
       </c>
       <c r="B37" s="56"/>
@@ -1621,7 +1621,7 @@
       <c r="F37" s="3"/>
     </row>
     <row r="38" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="65" t="s">
+      <c r="A38" s="57" t="s">
         <v>22</v>
       </c>
       <c r="B38" s="56"/>
@@ -1647,7 +1647,7 @@
       <c r="F40" s="2"/>
     </row>
     <row r="41" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="67" t="s">
+      <c r="A41" s="62" t="s">
         <v>23</v>
       </c>
       <c r="B41" s="56"/>
@@ -1665,7 +1665,7 @@
       <c r="F42" s="2"/>
     </row>
     <row r="43" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="64" t="s">
+      <c r="A43" s="55" t="s">
         <v>24</v>
       </c>
       <c r="B43" s="56"/>
@@ -2633,6 +2633,16 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A6:F6"/>
     <mergeCell ref="A43:F43"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A32:B32"/>
@@ -2648,16 +2658,6 @@
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A6:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2684,7 +2684,7 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="64" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
@@ -2694,7 +2694,7 @@
       <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="63" t="s">
         <v>25</v>
       </c>
       <c r="B3" s="56"/>
@@ -2720,7 +2720,7 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="67" t="s">
         <v>26</v>
       </c>
       <c r="B6" s="56"/>
@@ -2746,7 +2746,7 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="66" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="56"/>
@@ -2756,7 +2756,7 @@
       <c r="F9" s="56"/>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="69" t="s">
+      <c r="A10" s="68" t="s">
         <v>28</v>
       </c>
       <c r="B10" s="56"/>
@@ -2817,7 +2817,7 @@
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="61" t="s">
+      <c r="A16" s="66" t="s">
         <v>33</v>
       </c>
       <c r="B16" s="56"/>
@@ -2827,7 +2827,7 @@
       <c r="F16" s="56"/>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="69" t="s">
+      <c r="A17" s="68" t="s">
         <v>34</v>
       </c>
       <c r="B17" s="56"/>
@@ -2968,7 +2968,7 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="61" t="s">
+      <c r="A26" s="66" t="s">
         <v>48</v>
       </c>
       <c r="B26" s="56"/>
@@ -2978,7 +2978,7 @@
       <c r="F26" s="56"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="69" t="s">
+      <c r="A27" s="68" t="s">
         <v>49</v>
       </c>
       <c r="B27" s="56"/>
@@ -2996,7 +2996,7 @@
         <v>0</v>
       </c>
       <c r="C28" s="4"/>
-      <c r="D28" s="68" t="s">
+      <c r="D28" s="69" t="s">
         <v>51</v>
       </c>
       <c r="E28" s="56"/>
@@ -3011,7 +3011,7 @@
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="61" t="s">
+      <c r="A30" s="66" t="s">
         <v>52</v>
       </c>
       <c r="B30" s="56"/>
@@ -3021,7 +3021,7 @@
       <c r="F30" s="56"/>
     </row>
     <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="69" t="s">
+      <c r="A31" s="68" t="s">
         <v>53</v>
       </c>
       <c r="B31" s="56"/>
@@ -3053,7 +3053,7 @@
         <f>D21</f>
         <v>0</v>
       </c>
-      <c r="C33" s="68" t="s">
+      <c r="C33" s="69" t="s">
         <v>55</v>
       </c>
       <c r="D33" s="56"/>
@@ -3083,7 +3083,7 @@
         <f>B28</f>
         <v>0</v>
       </c>
-      <c r="C35" s="68" t="s">
+      <c r="C35" s="69" t="s">
         <v>60</v>
       </c>
       <c r="D35" s="56"/>
@@ -3099,7 +3099,7 @@
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="64" t="s">
+      <c r="A37" s="55" t="s">
         <v>24</v>
       </c>
       <c r="B37" s="56"/>
@@ -4073,6 +4073,13 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A37:F37"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="A27:F27"/>
@@ -4083,13 +4090,6 @@
     <mergeCell ref="C32:F32"/>
     <mergeCell ref="A30:F30"/>
     <mergeCell ref="A16:F16"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -4118,7 +4118,7 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="64" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
@@ -4128,7 +4128,7 @@
       <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="63" t="s">
         <v>61</v>
       </c>
       <c r="B3" s="56"/>
@@ -4154,7 +4154,7 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="67" t="s">
         <v>62</v>
       </c>
       <c r="B6" s="56"/>
@@ -4198,7 +4198,7 @@
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="66" t="s">
         <v>68</v>
       </c>
       <c r="B10" s="56"/>
@@ -4267,7 +4267,7 @@
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="61" t="s">
+      <c r="A15" s="66" t="s">
         <v>73</v>
       </c>
       <c r="B15" s="56"/>
@@ -4353,7 +4353,7 @@
       <c r="F20" s="2"/>
     </row>
     <row r="21" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="61" t="s">
+      <c r="A21" s="66" t="s">
         <v>79</v>
       </c>
       <c r="B21" s="56"/>
@@ -4420,7 +4420,7 @@
       <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="61" t="s">
+      <c r="A26" s="66" t="s">
         <v>84</v>
       </c>
       <c r="B26" s="56"/>
@@ -4489,7 +4489,7 @@
       <c r="F30" s="2"/>
     </row>
     <row r="31" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="66" t="s">
         <v>89</v>
       </c>
       <c r="B31" s="56"/>
@@ -4558,7 +4558,7 @@
       <c r="F35" s="2"/>
     </row>
     <row r="36" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="61" t="s">
+      <c r="A36" s="66" t="s">
         <v>94</v>
       </c>
       <c r="B36" s="56"/>
@@ -4650,7 +4650,7 @@
       <c r="F42" s="2"/>
     </row>
     <row r="43" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="61" t="s">
+      <c r="A43" s="66" t="s">
         <v>99</v>
       </c>
       <c r="B43" s="56"/>
@@ -4660,7 +4660,7 @@
       <c r="F43" s="56"/>
     </row>
     <row r="44" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="69" t="s">
+      <c r="A44" s="68" t="s">
         <v>100</v>
       </c>
       <c r="B44" s="56"/>
@@ -4677,7 +4677,7 @@
         <f>C41</f>
         <v>0</v>
       </c>
-      <c r="C45" s="68" t="s">
+      <c r="C45" s="69" t="s">
         <v>102</v>
       </c>
       <c r="D45" s="56"/>
@@ -4702,10 +4702,10 @@
         <v>104</v>
       </c>
       <c r="B47" s="38">
-        <f>IFERROR('Net Position Snapshot'!B12/C41,0)</f>
+        <f>IF(C41&gt;0, SUM(B11:B39)/(C41*12), 0)</f>
         <v>0</v>
       </c>
-      <c r="C47" s="68" t="s">
+      <c r="C47" s="69" t="s">
         <v>105</v>
       </c>
       <c r="D47" s="56"/>
@@ -4721,7 +4721,7 @@
       <c r="F48" s="2"/>
     </row>
     <row r="49" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="64" t="s">
+      <c r="A49" s="55" t="s">
         <v>24</v>
       </c>
       <c r="B49" s="56"/>
@@ -5725,7 +5725,7 @@
       <c r="F1" s="25"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="64" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
@@ -5735,7 +5735,7 @@
       <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="63" t="s">
         <v>106</v>
       </c>
       <c r="B3" s="56"/>
@@ -5761,7 +5761,7 @@
       <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="67" t="s">
         <v>107</v>
       </c>
       <c r="B6" s="56"/>
@@ -5803,7 +5803,7 @@
       <c r="F9" s="5"/>
     </row>
     <row r="10" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="66" t="s">
         <v>112</v>
       </c>
       <c r="B10" s="56"/>
@@ -5813,7 +5813,7 @@
       <c r="F10" s="56"/>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="69" t="s">
+      <c r="A11" s="68" t="s">
         <v>113</v>
       </c>
       <c r="B11" s="56"/>
@@ -5848,7 +5848,7 @@
       <c r="F13" s="5"/>
     </row>
     <row r="14" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="66" t="s">
         <v>116</v>
       </c>
       <c r="B14" s="56"/>
@@ -5858,7 +5858,7 @@
       <c r="F14" s="56"/>
     </row>
     <row r="15" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="69" t="s">
+      <c r="A15" s="68" t="s">
         <v>117</v>
       </c>
       <c r="B15" s="56"/>
@@ -5942,7 +5942,7 @@
       <c r="F21" s="5"/>
     </row>
     <row r="22" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="61" t="s">
+      <c r="A22" s="66" t="s">
         <v>124</v>
       </c>
       <c r="B22" s="56"/>
@@ -5952,7 +5952,7 @@
       <c r="F22" s="56"/>
     </row>
     <row r="23" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="69" t="s">
+      <c r="A23" s="68" t="s">
         <v>125</v>
       </c>
       <c r="B23" s="56"/>
@@ -6048,7 +6048,7 @@
       <c r="F30" s="5"/>
     </row>
     <row r="31" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="66" t="s">
         <v>133</v>
       </c>
       <c r="B31" s="56"/>
@@ -6058,7 +6058,7 @@
       <c r="F31" s="56"/>
     </row>
     <row r="32" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="69" t="s">
+      <c r="A32" s="68" t="s">
         <v>134</v>
       </c>
       <c r="B32" s="56"/>
@@ -6147,7 +6147,7 @@
       <c r="F38" s="5"/>
     </row>
     <row r="39" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="61" t="s">
+      <c r="A39" s="66" t="s">
         <v>143</v>
       </c>
       <c r="B39" s="56"/>
@@ -6157,7 +6157,7 @@
       <c r="F39" s="56"/>
     </row>
     <row r="40" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="69" t="s">
+      <c r="A40" s="68" t="s">
         <v>144</v>
       </c>
       <c r="B40" s="56"/>
@@ -6250,7 +6250,7 @@
       <c r="F46" s="2"/>
     </row>
     <row r="47" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="64" t="s">
+      <c r="A47" s="55" t="s">
         <v>24</v>
       </c>
       <c r="B47" s="56"/>
@@ -7255,7 +7255,7 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="64" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="56"/>
@@ -7265,7 +7265,7 @@
       <c r="F2" s="56"/>
     </row>
     <row r="3" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="63" t="s">
         <v>154</v>
       </c>
       <c r="B3" s="56"/>
@@ -7291,7 +7291,7 @@
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="63" t="s">
+      <c r="A6" s="67" t="s">
         <v>155</v>
       </c>
       <c r="B6" s="56"/>
@@ -7317,7 +7317,7 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="66" t="s">
         <v>156</v>
       </c>
       <c r="B9" s="56"/>
@@ -7345,7 +7345,7 @@
       <c r="B11" s="54">
         <v>0</v>
       </c>
-      <c r="C11" s="68" t="s">
+      <c r="C11" s="69" t="s">
         <v>160</v>
       </c>
       <c r="D11" s="56"/>
@@ -7373,7 +7373,7 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="61" t="s">
+      <c r="A14" s="66" t="s">
         <v>163</v>
       </c>
       <c r="B14" s="56"/>
@@ -7406,7 +7406,7 @@
       <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="61" t="s">
+      <c r="A17" s="66" t="s">
         <v>166</v>
       </c>
       <c r="B17" s="56"/>
@@ -7416,7 +7416,7 @@
       <c r="F17" s="56"/>
     </row>
     <row r="18" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="69" t="s">
+      <c r="A18" s="68" t="s">
         <v>167</v>
       </c>
       <c r="B18" s="56"/>
@@ -7430,7 +7430,7 @@
         <v>168</v>
       </c>
       <c r="B19" s="56"/>
-      <c r="C19" s="68" t="s">
+      <c r="C19" s="69" t="s">
         <v>169</v>
       </c>
       <c r="D19" s="56"/>
@@ -7440,7 +7440,7 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="75" t="s">
+      <c r="A20" s="73" t="s">
         <v>171</v>
       </c>
       <c r="B20" s="56"/>
@@ -7458,7 +7458,7 @@
         <v>173</v>
       </c>
       <c r="B21" s="56"/>
-      <c r="C21" s="68" t="s">
+      <c r="C21" s="69" t="s">
         <v>174</v>
       </c>
       <c r="D21" s="56"/>
@@ -7468,7 +7468,7 @@
       </c>
     </row>
     <row r="22" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="75" t="s">
+      <c r="A22" s="73" t="s">
         <v>175</v>
       </c>
       <c r="B22" s="56"/>
@@ -7486,7 +7486,7 @@
         <v>178</v>
       </c>
       <c r="B23" s="56"/>
-      <c r="C23" s="68" t="s">
+      <c r="C23" s="69" t="s">
         <v>179</v>
       </c>
       <c r="D23" s="56"/>
@@ -7496,7 +7496,7 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="75" t="s">
+      <c r="A24" s="73" t="s">
         <v>181</v>
       </c>
       <c r="B24" s="56"/>
@@ -7514,7 +7514,7 @@
         <v>184</v>
       </c>
       <c r="B25" s="56"/>
-      <c r="C25" s="68" t="s">
+      <c r="C25" s="69" t="s">
         <v>185</v>
       </c>
       <c r="D25" s="56"/>
@@ -7524,7 +7524,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="75" t="s">
+      <c r="A26" s="73" t="s">
         <v>187</v>
       </c>
       <c r="B26" s="56"/>
@@ -7546,7 +7546,7 @@
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="61" t="s">
+      <c r="A28" s="66" t="s">
         <v>190</v>
       </c>
       <c r="B28" s="56"/>
@@ -7560,7 +7560,7 @@
         <v>191</v>
       </c>
       <c r="B29" s="3"/>
-      <c r="C29" s="68" t="s">
+      <c r="C29" s="69" t="s">
         <v>192</v>
       </c>
       <c r="D29" s="56"/>
@@ -7584,7 +7584,7 @@
         <v>66</v>
       </c>
       <c r="B31" s="3"/>
-      <c r="C31" s="68"/>
+      <c r="C31" s="69"/>
       <c r="D31" s="56"/>
       <c r="E31" s="56"/>
       <c r="F31" s="56"/>
@@ -7598,7 +7598,7 @@
       <c r="F32" s="2"/>
     </row>
     <row r="33" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="73" t="s">
+      <c r="A33" s="75" t="s">
         <v>195</v>
       </c>
       <c r="B33" s="56"/>
@@ -7616,7 +7616,7 @@
       <c r="F34" s="2"/>
     </row>
     <row r="35" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="64" t="s">
+      <c r="A35" s="55" t="s">
         <v>24</v>
       </c>
       <c r="B35" s="56"/>
@@ -8592,6 +8592,23 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C22:E22"/>
     <mergeCell ref="C25:E25"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A35:F35"/>
@@ -8608,23 +8625,6 @@
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="A33:F33"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="A18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>